<commit_message>
I Love It: drei Blinder nach Änderungswunsch
- youre on a different road: starker Blinder auf der letzten Viertel (Snarewirbel)
- STOP: kurzer Blinder auf die Eins, danach schwarz
- chorus 4: Blinder auf den Einsatz

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/songs/ILoveIt_v1/quelle/struktur.xlsx
+++ b/songs/ILoveIt_v1/quelle/struktur.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\00_DATEN\PlatformIO\Projects\LED-GIT_on_YULC\songs\ILoveIt_v1\quelle\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B74B9C6E-2C7F-4153-B182-6C26243E068E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA5912D3-6F8F-4AD9-8F79-6B7FAF88DC61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1644" yWindow="11412" windowWidth="27648" windowHeight="12276" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9936" yWindow="12864" windowWidth="27648" windowHeight="12276" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Struktur" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="57">
   <si>
     <t>I Love It</t>
   </si>
@@ -138,7 +138,8 @@
   </si>
   <si>
     <t>progPalette(16000, 11, 35)
-Alter Effekt: grüner Verlauf, der zu Weiß aufhellt.</t>
+Ausgabe: Blinder bei 15500 ms, 1000 ms lang, Blinder blendet 0 ms ein, 500 ms voll, 500 ms aus
+Alter Effekt: grüner Verlauf, der zu Weiß aufhellt. Auf der letzten Viertel (Snarewirbel) ein starker Blinder, der bis zum Part-Ende voll steht.</t>
   </si>
   <si>
     <t>progPalette(16000, 11, 35)</t>
@@ -185,7 +186,8 @@
   </si>
   <si>
     <t>progBlack(2000, 60)
-Alter Effekt: 1 Takt schwarz.</t>
+Ausgabe: Blinder bei 0 ms, 500 ms lang
+Kurzer Blinder auf die Eins, der in einem Beat abklingt - danach der Rest des Takts schwarz.</t>
   </si>
   <si>
     <t>progBlack(2000, 60)</t>
@@ -195,7 +197,8 @@
   </si>
   <si>
     <t>progSternNeu(16000, 500, 65, 5, 26, 5, false, 4)
-Alter Effekt: drehender Stern, fest in der Mitte, Farbwechsel pro Beat.</t>
+Ausgabe: Blinder bei 0 ms, 1000 ms lang
+Blinder auf den Einsatz (klingt über 2 Beats ab), darunter der alte Effekt: drehender Stern, fest in der Mitte, Farbwechsel pro Beat.</t>
   </si>
   <si>
     <t>progSternNeu(16000, 500, 65, 5, 26, 5, false, 4)</t>
@@ -217,13 +220,10 @@
     <t>10 sek. BLACK</t>
   </si>
   <si>
-    <t>kurzer blinder vor der BLACK phase</t>
-  </si>
-  <si>
-    <t>blinder am anfang</t>
-  </si>
-  <si>
-    <t>am ende auf der letzten viertel starker BLINDER (auf snarewirbel)</t>
+    <t>der blinder am ende wikrt nicht! Zu wenig sichtbares reinblenden und zu kurz</t>
+  </si>
+  <si>
+    <t>Starker blinder am ende</t>
   </si>
 </sst>
 </file>
@@ -659,7 +659,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4">
         <v>0</v>
       </c>
@@ -679,7 +679,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <v>3</v>
       </c>
@@ -699,7 +699,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>7</v>
       </c>
@@ -719,7 +719,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4">
         <v>15</v>
       </c>
@@ -739,7 +739,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4">
         <v>19</v>
       </c>
@@ -759,7 +759,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4">
         <v>27</v>
       </c>
@@ -779,7 +779,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4">
         <v>31</v>
       </c>
@@ -790,7 +790,7 @@
         <v>31</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E12" s="5"/>
       <c r="F12" s="5">
@@ -801,7 +801,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4">
         <v>39</v>
       </c>
@@ -821,7 +821,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
         <v>47</v>
       </c>
@@ -841,7 +841,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4">
         <v>55</v>
       </c>
@@ -861,7 +861,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4">
         <v>63</v>
       </c>
@@ -881,7 +881,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4">
         <v>70</v>
       </c>
@@ -891,9 +891,7 @@
       <c r="C17" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="D17" s="6" t="s">
-        <v>55</v>
-      </c>
+      <c r="D17" s="6"/>
       <c r="E17" s="5"/>
       <c r="F17" s="5">
         <f t="shared" si="0"/>
@@ -903,7 +901,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
         <v>71</v>
       </c>
@@ -913,9 +911,7 @@
       <c r="C18" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="D18" s="6" t="s">
-        <v>56</v>
-      </c>
+      <c r="D18" s="6"/>
       <c r="E18" s="5"/>
       <c r="F18" s="5">
         <f t="shared" si="0"/>
@@ -925,7 +921,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4">
         <v>79</v>
       </c>
@@ -935,7 +931,9 @@
       <c r="C19" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D19" s="6"/>
+      <c r="D19" s="6" t="s">
+        <v>56</v>
+      </c>
       <c r="E19" s="5"/>
       <c r="F19" s="5">
         <f t="shared" si="0"/>

</xml_diff>